<commit_message>
finish purchases & Suppliers section
</commit_message>
<xml_diff>
--- a/fatorize_erp_system/SQL Scripts/نموذج جدول بنود الفاتورة وجدول مبالغ الفاتورة.xlsx
+++ b/fatorize_erp_system/SQL Scripts/نموذج جدول بنود الفاتورة وجدول مبالغ الفاتورة.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\fatorize_erp_system\SQL Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE8F6B8B-97B7-496E-A94F-EBC7C7AC12AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9761235B-80B0-4253-BF66-177C36794D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD2D17FE-759C-434D-9D0D-A2F4EB1D6AB0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AD2D17FE-759C-434D-9D0D-A2F4EB1D6AB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
   <si>
     <t>عملة الفاتورة</t>
   </si>
@@ -104,9 +105,6 @@
     <t>الكروب / القياس</t>
   </si>
   <si>
-    <t>عدد القطع بالباكيت</t>
-  </si>
-  <si>
     <t xml:space="preserve">اللون </t>
   </si>
   <si>
@@ -116,22 +114,19 @@
     <t>عدد المنتجات</t>
   </si>
   <si>
-    <t>نسبة الخصم اللإفرادي</t>
-  </si>
-  <si>
-    <t>الاجمالي (بعملة الفرع)</t>
-  </si>
-  <si>
-    <t>الاجمالي (بعملة الفاتورة)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> سعر الوحدة الافتراضي بعملة الفرع</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> سعر الوحدة الافتراضي بعملة الفاتورة</t>
-  </si>
-  <si>
-    <t>سعرالوحدة بعد الخصم الافرادي بعملة الفاتورة</t>
+    <t xml:space="preserve"> سعر البيع الافتراضي selling_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قيمة الخصم الإفرادي discount_amount </t>
+  </si>
+  <si>
+    <t>سعرالبيع بعد الخصم الافرادي</t>
+  </si>
+  <si>
+    <t>عدد القطع بالباكيت packet_qty</t>
+  </si>
+  <si>
+    <t>الاجمالي</t>
   </si>
 </sst>
 </file>
@@ -235,16 +230,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -581,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{891B50B3-7E85-41EA-B516-8EB370A41949}">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57" style="1" bestFit="1" customWidth="1"/>
@@ -605,22 +600,22 @@
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
     </row>
     <row r="4" spans="1:3" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -669,7 +664,7 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="5"/>
@@ -678,7 +673,7 @@
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="5"/>
@@ -709,7 +704,7 @@
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="5"/>
@@ -736,77 +731,95 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="5"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A17:N17"/>
+  <mergeCells count="6">
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B13:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52DF6317-A910-4C01-8BD4-BC9F2F6F3E7D}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+    </row>
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>